<commit_message>
update templates/* amd README.md
</commit_message>
<xml_diff>
--- a/templates/check_iot_ai.xlsx
+++ b/templates/check_iot_ai.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AutoReport_AI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AutoReport_AI\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{727EEB9B-3B83-428F-AD05-4BFDE2E142E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C944F09-49CA-44EE-9E93-ADEDA3CB1EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="15" windowWidth="29040" windowHeight="15720" tabRatio="426" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -164,23 +164,6 @@
     <t>Low</t>
   </si>
   <si>
-    <t>測試方式：
-- 進行藍牙通訊側錄與配對流程確認，並參考「藍牙5.1 CVE list」分頁檢視相關公開弱點資訊。
-測試結果：
-- 藍牙版本為 5.1。
-- 傳輸過程有啟用加密。
-- 裝置發起配對時採 Just Works 模式，不需輸入 PIN Code／Passkey。
-- 「藍牙5.1 CVE list」分頁包含高風險項目，實際適用性仍需依使用之藍牙堆疊、實作與版本確認。
-攻擊條件：
-- 攻擊者需位於藍牙通訊範圍內。
-- 裝置藍牙需由使用者按下實體按鈕後人工啟動，並非長時間持續開啟。
-可能影響：
-- Just Works 配對不要求 PIN Code／Passkey；若相關配對或藍牙協定弱點適用，可能存在未經充分身分驗證之配對、通訊攔截或資料遭未授權存取的風險。
-既有防護／限制條件：
-- 藍牙由裝置實體按鈕人工啟動，非長時間開啟。
-- 傳輸敏感性資料時已有加密保護。</t>
-  </si>
-  <si>
     <t>P07          </t>
   </si>
   <si>
@@ -193,37 +176,10 @@
     <t>Sensitive Data Leakage</t>
   </si>
   <si>
-    <t>測試方式：
-- 確認敏感性資料之傳輸方式與傳輸保護情形，並參考 P06 藍牙測試結果。
-測試結果：
-- 資料僅透過藍牙傳輸，藍牙傳輸時資料有加密。
-攻擊條件：
-- 需位於藍牙通訊範圍內，且在裝置藍牙啟用期間進行攻擊；其他配對條件參考 P06。
-可能影響：
-- 若藍牙配對或傳輸保護機制遭利用，可能造成敏感性資料遭未授權存取或暴露。
-既有防護／限制條件：
-- 敏感性資料傳輸已有加密保護。
-- 藍牙非長時間開啟，啟用條件參考 P06。</t>
-  </si>
-  <si>
     <t>P09          </t>
   </si>
   <si>
     <t>API Authentication</t>
-  </si>
-  <si>
-    <t>測試方式：
-- 本測項依 P06 所述藍牙配對與連線機制進行判定。
-測試結果：
-- 參考 P06：裝置採 Just Works 配對模式，不需輸入 PIN Code／Passkey。
-- 原始資料未另外提供獨立 API 驗證流程或介面細節。
-攻擊條件：
-- 需位於藍牙通訊範圍內，且裝置需處於藍牙啟用／配對情境；其他條件參考 P06。
-可能影響：
-- 在 Just Works 配對情境下，身分確認能力較有限，可能存在未經充分驗證之存取風險；實際 API 權限與可存取範圍仍需依產品實作確認。
-既有防護／限制條件：
-- 藍牙由裝置實體按鈕人工啟動，非長時間開啟。
-- 傳輸敏感性資料時已有加密保護，相關內容參考 P06。</t>
   </si>
   <si>
     <t>P10          </t>
@@ -1102,6 +1058,53 @@
 既有防護／限制條件：
 - 已提供 Read Protection 防止韌體讀取。</t>
     </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>測試方式：
+- 進行藍牙通訊側錄與配對流程確認，並參考「藍牙5.1 CVE list」分頁檢視相關公開弱點資訊。
+測試結果：
+- 藍牙版本為 5.1。
+- 傳輸過程有啟用加密。
+- 裝置發起配對時採 Just Works 模式，不需輸入 PIN Code／Passkey。
+- 「藍牙5.1 CVE list」分頁包含高風險項目，實際適用性仍需依使用之藍牙堆疊、實作與版本確認。
+攻擊條件：
+- 攻擊者需位於藍牙通訊範圍內。
+- 裝置藍牙需由使用者按下實體按鈕後人工啟動，並非長時間持續開啟。
+可能影響：
+- Just Works 配對不要求 PIN Code／Passkey；若相關配對或藍牙協定弱點適用，可能存在未經充分身分驗證之配對、通訊攔截或資料遭未授權存取的風險。
+既有防護／限制條件：
+- 藍牙由裝置實體按鈕人工啟動，非長時間開啟。
+- 傳輸敏感性資料時已有加密保護。</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>測試方式：
+- 確認敏感性資料之傳輸方式與傳輸保護情形，並參考 P06 藍牙測試結果。
+測試結果：
+- 資料僅透過藍牙傳輸，藍牙傳輸時資料有加密。
+攻擊條件：
+- 需位於藍牙通訊範圍內，且在裝置藍牙啟用期間進行攻擊；其他配對條件參考 P06。
+可能影響：
+- 若藍牙配對或傳輸保護機制遭利用，可能造成敏感性資料遭未授權存取或暴露。
+既有防護／限制條件：
+- 敏感性資料傳輸已有加密保護。
+- 藍牙非長時間開啟，啟用條件參考 P06。</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>測試方式：
+- 本測項依 P06 所述藍牙配對與連線機制進行判定。
+測試結果：
+- 參考 P06：裝置採 Just Works 配對模式，不需輸入 PIN Code／Passkey。
+- 原始資料未另外提供獨立 API 驗證流程或介面細節。
+攻擊條件：
+- 需位於藍牙通訊範圍內，且裝置需處於藍牙啟用／配對情境；其他條件參考 P06。
+可能影響：
+- 在 Just Works 配對情境下，身分確認能力較有限，可能存在未經充分驗證之存取風險；實際 API 權限與可存取範圍仍需依產品實作確認。
+既有防護／限制條件：
+- 藍牙由裝置實體按鈕人工啟動，非長時間開啟。
+- 傳輸敏感性資料時已有加密保護，相關內容參考 P06。</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -1575,9 +1578,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="15" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1678,6 +1678,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
@@ -1979,41 +1982,41 @@
     <col min="14" max="16384" width="8.69140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="63" customFormat="1" ht="26.6" customHeight="1">
-      <c r="A1" s="61" t="s">
+    <row r="1" spans="1:12" s="62" customFormat="1" ht="26.6" customHeight="1">
+      <c r="A1" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="61" t="s">
+      <c r="B1" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="61" t="s">
+      <c r="C1" s="60" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="61" t="s">
+      <c r="D1" s="60" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="62" t="s">
+      <c r="E1" s="61" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="62" t="s">
+      <c r="F1" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="62" t="s">
+      <c r="G1" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="62" t="s">
+      <c r="H1" s="61" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="62" t="s">
+      <c r="I1" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="62" t="s">
+      <c r="J1" s="61" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="62" t="s">
+      <c r="K1" s="61" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="62" t="s">
+      <c r="L1" s="61" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2027,19 +2030,19 @@
       <c r="C2" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="25" t="s">
-        <v>164</v>
-      </c>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="J2" s="25"/>
-      <c r="K2" s="25"/>
-      <c r="L2" s="25"/>
+      <c r="E2" s="63" t="s">
+        <v>161</v>
+      </c>
+      <c r="F2" s="63"/>
+      <c r="G2" s="63"/>
+      <c r="H2" s="63"/>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
+      <c r="K2" s="63"/>
+      <c r="L2" s="63"/>
     </row>
     <row r="3" spans="1:12" ht="200.05" customHeight="1">
       <c r="A3" s="15" t="s">
@@ -2051,19 +2054,19 @@
       <c r="C3" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="25" t="s">
-        <v>165</v>
-      </c>
-      <c r="F3" s="25"/>
-      <c r="G3" s="25"/>
-      <c r="H3" s="25"/>
-      <c r="I3" s="25"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
+      <c r="E3" s="63" t="s">
+        <v>162</v>
+      </c>
+      <c r="F3" s="63"/>
+      <c r="G3" s="63"/>
+      <c r="H3" s="63"/>
+      <c r="I3" s="63"/>
+      <c r="J3" s="63"/>
+      <c r="K3" s="63"/>
+      <c r="L3" s="63"/>
     </row>
     <row r="4" spans="1:12" ht="200.05" customHeight="1">
       <c r="A4" s="17" t="s">
@@ -2075,19 +2078,19 @@
       <c r="C4" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="25" t="s">
-        <v>166</v>
-      </c>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
-      <c r="J4" s="25"/>
-      <c r="K4" s="25"/>
-      <c r="L4" s="25"/>
+      <c r="E4" s="63" t="s">
+        <v>163</v>
+      </c>
+      <c r="F4" s="63"/>
+      <c r="G4" s="63"/>
+      <c r="H4" s="63"/>
+      <c r="I4" s="63"/>
+      <c r="J4" s="63"/>
+      <c r="K4" s="63"/>
+      <c r="L4" s="63"/>
     </row>
     <row r="5" spans="1:12" ht="200.05" customHeight="1">
       <c r="A5" s="19" t="s">
@@ -2099,19 +2102,19 @@
       <c r="C5" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="25" t="s">
-        <v>167</v>
-      </c>
-      <c r="F5" s="25"/>
-      <c r="G5" s="25"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-      <c r="K5" s="25"/>
-      <c r="L5" s="25"/>
+      <c r="E5" s="63" t="s">
+        <v>164</v>
+      </c>
+      <c r="F5" s="63"/>
+      <c r="G5" s="63"/>
+      <c r="H5" s="63"/>
+      <c r="I5" s="63"/>
+      <c r="J5" s="63"/>
+      <c r="K5" s="63"/>
+      <c r="L5" s="63"/>
     </row>
     <row r="6" spans="1:12" ht="200.05" customHeight="1">
       <c r="A6" s="21" t="s">
@@ -2123,19 +2126,19 @@
       <c r="C6" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="25" t="s">
-        <v>168</v>
-      </c>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
-      <c r="J6" s="25"/>
-      <c r="K6" s="25"/>
-      <c r="L6" s="25"/>
+      <c r="E6" s="63" t="s">
+        <v>165</v>
+      </c>
+      <c r="F6" s="63"/>
+      <c r="G6" s="63"/>
+      <c r="H6" s="63"/>
+      <c r="I6" s="63"/>
+      <c r="J6" s="63"/>
+      <c r="K6" s="63"/>
+      <c r="L6" s="63"/>
     </row>
     <row r="7" spans="1:12" ht="200.05" customHeight="1">
       <c r="A7" s="21" t="s">
@@ -2147,19 +2150,19 @@
       <c r="C7" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="25" t="s">
-        <v>169</v>
-      </c>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="25"/>
-      <c r="L7" s="25"/>
+      <c r="E7" s="63" t="s">
+        <v>166</v>
+      </c>
+      <c r="F7" s="63"/>
+      <c r="G7" s="63"/>
+      <c r="H7" s="63"/>
+      <c r="I7" s="63"/>
+      <c r="J7" s="63"/>
+      <c r="K7" s="63"/>
+      <c r="L7" s="63"/>
     </row>
     <row r="8" spans="1:12" ht="200.05" customHeight="1">
       <c r="A8" s="21" t="s">
@@ -2171,19 +2174,19 @@
       <c r="C8" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="25" t="s">
-        <v>170</v>
-      </c>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
-      <c r="J8" s="25"/>
-      <c r="K8" s="25"/>
-      <c r="L8" s="25"/>
+      <c r="E8" s="63" t="s">
+        <v>167</v>
+      </c>
+      <c r="F8" s="63"/>
+      <c r="G8" s="63"/>
+      <c r="H8" s="63"/>
+      <c r="I8" s="63"/>
+      <c r="J8" s="63"/>
+      <c r="K8" s="63"/>
+      <c r="L8" s="63"/>
     </row>
     <row r="9" spans="1:12" ht="200.05" customHeight="1">
       <c r="A9" s="21" t="s">
@@ -2195,19 +2198,19 @@
       <c r="C9" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="25" t="s">
-        <v>171</v>
-      </c>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
-      <c r="J9" s="25"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25"/>
+      <c r="E9" s="63" t="s">
+        <v>168</v>
+      </c>
+      <c r="F9" s="63"/>
+      <c r="G9" s="63"/>
+      <c r="H9" s="63"/>
+      <c r="I9" s="63"/>
+      <c r="J9" s="63"/>
+      <c r="K9" s="63"/>
+      <c r="L9" s="63"/>
     </row>
     <row r="10" spans="1:12" ht="200.05" customHeight="1">
       <c r="A10" s="21" t="s">
@@ -2219,19 +2222,19 @@
       <c r="C10" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="25" t="s">
-        <v>172</v>
-      </c>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="25"/>
-      <c r="J10" s="25"/>
-      <c r="K10" s="25"/>
-      <c r="L10" s="25"/>
+      <c r="E10" s="63" t="s">
+        <v>169</v>
+      </c>
+      <c r="F10" s="63"/>
+      <c r="G10" s="63"/>
+      <c r="H10" s="63"/>
+      <c r="I10" s="63"/>
+      <c r="J10" s="63"/>
+      <c r="K10" s="63"/>
+      <c r="L10" s="63"/>
     </row>
     <row r="11" spans="1:12" ht="200.05" customHeight="1">
       <c r="A11" s="21" t="s">
@@ -2243,355 +2246,355 @@
       <c r="C11" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="25"/>
+      <c r="E11" s="63" t="s">
+        <v>182</v>
+      </c>
+      <c r="F11" s="63"/>
+      <c r="G11" s="63"/>
+      <c r="H11" s="63"/>
+      <c r="I11" s="63"/>
+      <c r="J11" s="63"/>
+      <c r="K11" s="63"/>
+      <c r="L11" s="63"/>
     </row>
     <row r="12" spans="1:12" ht="200.05" customHeight="1">
       <c r="A12" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B12" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="25" t="s">
-        <v>173</v>
-      </c>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
+      <c r="E12" s="63" t="s">
+        <v>170</v>
+      </c>
+      <c r="F12" s="63"/>
+      <c r="G12" s="63"/>
+      <c r="H12" s="63"/>
+      <c r="I12" s="63"/>
+      <c r="J12" s="63"/>
+      <c r="K12" s="63"/>
+      <c r="L12" s="63"/>
     </row>
     <row r="13" spans="1:12" ht="200.05" customHeight="1">
       <c r="A13" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B13" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" s="26" t="s">
+      <c r="D13" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="E13" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25"/>
-      <c r="L13" s="25"/>
+      <c r="E13" s="63" t="s">
+        <v>183</v>
+      </c>
+      <c r="F13" s="63"/>
+      <c r="G13" s="63"/>
+      <c r="H13" s="63"/>
+      <c r="I13" s="63"/>
+      <c r="J13" s="63"/>
+      <c r="K13" s="63"/>
+      <c r="L13" s="63"/>
     </row>
     <row r="14" spans="1:12" ht="200.05" customHeight="1">
       <c r="A14" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
-      <c r="I14" s="25"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25"/>
-      <c r="L14" s="25"/>
+      <c r="E14" s="63" t="s">
+        <v>184</v>
+      </c>
+      <c r="F14" s="63"/>
+      <c r="G14" s="63"/>
+      <c r="H14" s="63"/>
+      <c r="I14" s="63"/>
+      <c r="J14" s="63"/>
+      <c r="K14" s="63"/>
+      <c r="L14" s="63"/>
     </row>
     <row r="15" spans="1:12" ht="200.05" customHeight="1">
       <c r="A15" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B15" s="22" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>49</v>
-      </c>
-      <c r="D15" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E15" s="25" t="s">
-        <v>174</v>
-      </c>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="25"/>
+      <c r="E15" s="63" t="s">
+        <v>171</v>
+      </c>
+      <c r="F15" s="63"/>
+      <c r="G15" s="63"/>
+      <c r="H15" s="63"/>
+      <c r="I15" s="63"/>
+      <c r="J15" s="63"/>
+      <c r="K15" s="63"/>
+      <c r="L15" s="63"/>
     </row>
     <row r="16" spans="1:12" ht="200.05" customHeight="1">
       <c r="A16" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="D16" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="25" t="s">
-        <v>175</v>
-      </c>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="25"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25"/>
-      <c r="L16" s="25"/>
+      <c r="E16" s="63" t="s">
+        <v>172</v>
+      </c>
+      <c r="F16" s="63"/>
+      <c r="G16" s="63"/>
+      <c r="H16" s="63"/>
+      <c r="I16" s="63"/>
+      <c r="J16" s="63"/>
+      <c r="K16" s="63"/>
+      <c r="L16" s="63"/>
     </row>
     <row r="17" spans="1:12" ht="200.05" customHeight="1">
       <c r="A17" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B17" s="22" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>53</v>
-      </c>
-      <c r="D17" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="25" t="s">
-        <v>176</v>
-      </c>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="25"/>
+      <c r="E17" s="63" t="s">
+        <v>173</v>
+      </c>
+      <c r="F17" s="63"/>
+      <c r="G17" s="63"/>
+      <c r="H17" s="63"/>
+      <c r="I17" s="63"/>
+      <c r="J17" s="63"/>
+      <c r="K17" s="63"/>
+      <c r="L17" s="63"/>
     </row>
     <row r="18" spans="1:12" ht="200.05" customHeight="1">
       <c r="A18" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="D18" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="25" t="s">
-        <v>177</v>
-      </c>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
-      <c r="I18" s="25"/>
-      <c r="J18" s="25"/>
-      <c r="K18" s="25"/>
-      <c r="L18" s="25"/>
+      <c r="E18" s="63" t="s">
+        <v>174</v>
+      </c>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="63"/>
+      <c r="I18" s="63"/>
+      <c r="J18" s="63"/>
+      <c r="K18" s="63"/>
+      <c r="L18" s="63"/>
     </row>
     <row r="19" spans="1:12" ht="200.05" customHeight="1">
       <c r="A19" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="D19" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E19" s="25" t="s">
-        <v>178</v>
-      </c>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
-      <c r="I19" s="25"/>
-      <c r="J19" s="25"/>
-      <c r="K19" s="25"/>
-      <c r="L19" s="25"/>
+      <c r="E19" s="63" t="s">
+        <v>175</v>
+      </c>
+      <c r="F19" s="63"/>
+      <c r="G19" s="63"/>
+      <c r="H19" s="63"/>
+      <c r="I19" s="63"/>
+      <c r="J19" s="63"/>
+      <c r="K19" s="63"/>
+      <c r="L19" s="63"/>
     </row>
     <row r="20" spans="1:12" ht="200.05" customHeight="1">
       <c r="A20" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="D20" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="25" t="s">
-        <v>179</v>
-      </c>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
-      <c r="L20" s="25"/>
+      <c r="E20" s="63" t="s">
+        <v>176</v>
+      </c>
+      <c r="F20" s="63"/>
+      <c r="G20" s="63"/>
+      <c r="H20" s="63"/>
+      <c r="I20" s="63"/>
+      <c r="J20" s="63"/>
+      <c r="K20" s="63"/>
+      <c r="L20" s="63"/>
     </row>
     <row r="21" spans="1:12" ht="200.05" customHeight="1">
       <c r="A21" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B21" s="22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>61</v>
-      </c>
-      <c r="D21" s="26" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E21" s="25" t="s">
-        <v>180</v>
-      </c>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="25"/>
-      <c r="J21" s="25"/>
-      <c r="K21" s="25"/>
-      <c r="L21" s="25"/>
+      <c r="E21" s="63" t="s">
+        <v>177</v>
+      </c>
+      <c r="F21" s="63"/>
+      <c r="G21" s="63"/>
+      <c r="H21" s="63"/>
+      <c r="I21" s="63"/>
+      <c r="J21" s="63"/>
+      <c r="K21" s="63"/>
+      <c r="L21" s="63"/>
     </row>
     <row r="22" spans="1:12" ht="200.05" customHeight="1">
       <c r="A22" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>63</v>
-      </c>
-      <c r="D22" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="D22" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E22" s="25" t="s">
-        <v>181</v>
-      </c>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="25"/>
-      <c r="J22" s="25"/>
-      <c r="K22" s="25"/>
-      <c r="L22" s="25"/>
+      <c r="E22" s="63" t="s">
+        <v>178</v>
+      </c>
+      <c r="F22" s="63"/>
+      <c r="G22" s="63"/>
+      <c r="H22" s="63"/>
+      <c r="I22" s="63"/>
+      <c r="J22" s="63"/>
+      <c r="K22" s="63"/>
+      <c r="L22" s="63"/>
     </row>
     <row r="23" spans="1:12" ht="200.05" customHeight="1">
       <c r="A23" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="22" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="D23" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="D23" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E23" s="25" t="s">
-        <v>182</v>
-      </c>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="25"/>
-      <c r="J23" s="25"/>
-      <c r="K23" s="25"/>
-      <c r="L23" s="25"/>
+      <c r="E23" s="63" t="s">
+        <v>179</v>
+      </c>
+      <c r="F23" s="63"/>
+      <c r="G23" s="63"/>
+      <c r="H23" s="63"/>
+      <c r="I23" s="63"/>
+      <c r="J23" s="63"/>
+      <c r="K23" s="63"/>
+      <c r="L23" s="63"/>
     </row>
     <row r="24" spans="1:12" ht="200.05" customHeight="1">
       <c r="A24" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B24" s="22" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>67</v>
-      </c>
-      <c r="D24" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E24" s="25" t="s">
-        <v>183</v>
-      </c>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="25"/>
-      <c r="J24" s="25"/>
-      <c r="K24" s="25"/>
-      <c r="L24" s="25"/>
+      <c r="E24" s="63" t="s">
+        <v>180</v>
+      </c>
+      <c r="F24" s="63"/>
+      <c r="G24" s="63"/>
+      <c r="H24" s="63"/>
+      <c r="I24" s="63"/>
+      <c r="J24" s="63"/>
+      <c r="K24" s="63"/>
+      <c r="L24" s="63"/>
     </row>
     <row r="25" spans="1:12" ht="200.05" customHeight="1">
       <c r="A25" s="21" t="s">
         <v>25</v>
       </c>
       <c r="B25" s="22" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="D25" s="26" t="s">
+        <v>66</v>
+      </c>
+      <c r="D25" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="E25" s="25" t="s">
-        <v>184</v>
-      </c>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
-      <c r="I25" s="25"/>
-      <c r="J25" s="25"/>
-      <c r="K25" s="25"/>
-      <c r="L25" s="25"/>
+      <c r="E25" s="63" t="s">
+        <v>181</v>
+      </c>
+      <c r="F25" s="63"/>
+      <c r="G25" s="63"/>
+      <c r="H25" s="63"/>
+      <c r="I25" s="63"/>
+      <c r="J25" s="63"/>
+      <c r="K25" s="63"/>
+      <c r="L25" s="63"/>
     </row>
     <row r="26" spans="1:12">
       <c r="B26" s="7"/>
@@ -2601,7 +2604,7 @@
     <row r="27" spans="1:12" ht="15.45" customHeight="1">
       <c r="D27" s="12"/>
       <c r="E27" s="9"/>
-      <c r="F27" s="31"/>
+      <c r="F27" s="30"/>
       <c r="G27" s="9"/>
     </row>
     <row r="28" spans="1:12" ht="15.45" customHeight="1">
@@ -9962,57 +9965,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="28" customHeight="1">
-      <c r="A1" s="58" t="s">
+      <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="58" t="s">
+      <c r="B1" s="57" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1" s="57" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1" s="57" t="s">
+        <v>69</v>
+      </c>
+      <c r="E1" s="57" t="s">
         <v>70</v>
       </c>
-      <c r="C1" s="58" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" s="58" t="s">
-        <v>72</v>
-      </c>
-      <c r="E1" s="58" t="s">
-        <v>73</v>
-      </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="59"/>
-      <c r="C2" s="59"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="59"/>
-      <c r="C3" s="59"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="59" t="s">
+      <c r="A4" s="58" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="59"/>
-      <c r="C4" s="59"/>
-      <c r="D4" s="60"/>
-      <c r="E4" s="60"/>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="59"/>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="59" t="s">
+      <c r="A5" s="58" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="59"/>
-      <c r="C5" s="59"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="60"/>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E5" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
@@ -10043,84 +10046,84 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="18.45" customHeight="1">
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="29" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="28"/>
+    </row>
+    <row r="2" spans="2:13" ht="15.9" customHeight="1">
+      <c r="B2" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="35" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="35" t="s">
         <v>74</v>
       </c>
-      <c r="D1" s="29"/>
-    </row>
-    <row r="2" spans="2:13" ht="15.9" customHeight="1">
-      <c r="B2" s="36" t="s">
+      <c r="E2" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="36" t="s">
+      <c r="F2" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="D2" s="36" t="s">
+      <c r="G2" s="36" t="s">
         <v>77</v>
       </c>
-      <c r="E2" s="37" t="s">
+      <c r="H2" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="F2" s="37" t="s">
+      <c r="I2" s="36" t="s">
         <v>79</v>
       </c>
-      <c r="G2" s="37" t="s">
+      <c r="J2" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="H2" s="37" t="s">
+      <c r="K2" s="36" t="s">
         <v>81</v>
       </c>
-      <c r="I2" s="37" t="s">
+      <c r="L2" s="35" t="s">
+        <v>7</v>
+      </c>
+      <c r="M2" s="27"/>
+    </row>
+    <row r="3" spans="2:13" ht="18" customHeight="1">
+      <c r="B3" s="31"/>
+      <c r="C3" s="32" t="s">
         <v>82</v>
       </c>
-      <c r="J2" s="37" t="s">
+      <c r="D3" s="33"/>
+      <c r="E3" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="K2" s="37" t="s">
+      <c r="F3" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="L2" s="36" t="s">
-        <v>7</v>
-      </c>
-      <c r="M2" s="28"/>
-    </row>
-    <row r="3" spans="2:13" ht="18" customHeight="1">
-      <c r="B3" s="32"/>
-      <c r="C3" s="33" t="s">
+      <c r="G3" s="33"/>
+      <c r="H3" s="33"/>
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33"/>
+      <c r="L3" s="33"/>
+    </row>
+    <row r="4" spans="2:13" ht="18" customHeight="1">
+      <c r="B4" s="31"/>
+      <c r="C4" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34" t="s">
-        <v>86</v>
-      </c>
-      <c r="F3" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
-      <c r="L3" s="34"/>
-    </row>
-    <row r="4" spans="2:13" ht="18" customHeight="1">
-      <c r="B4" s="32"/>
-      <c r="C4" s="33" t="s">
-        <v>85</v>
-      </c>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34" t="s">
-        <v>88</v>
-      </c>
-      <c r="F4" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="34"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="34"/>
+      <c r="F4" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="G4" s="33"/>
+      <c r="H4" s="33"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="33"/>
+      <c r="K4" s="33"/>
+      <c r="L4" s="33"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -10133,423 +10136,423 @@
   <dimension ref="A1:I17"/>
   <sheetFormatPr defaultColWidth="8.69140625" defaultRowHeight="12.9"/>
   <cols>
-    <col min="1" max="1" width="12.23046875" style="51" customWidth="1"/>
-    <col min="2" max="2" width="46.53515625" style="51" customWidth="1"/>
-    <col min="3" max="3" width="22.4609375" style="51" customWidth="1"/>
-    <col min="4" max="4" width="8.4609375" style="51" customWidth="1"/>
-    <col min="5" max="5" width="43.53515625" style="51" customWidth="1"/>
-    <col min="6" max="6" width="50.4609375" style="51" customWidth="1"/>
-    <col min="7" max="7" width="23.84375" style="51" customWidth="1"/>
-    <col min="8" max="8" width="54.4609375" style="51" customWidth="1"/>
-    <col min="9" max="9" width="20.15234375" style="57" customWidth="1"/>
-    <col min="10" max="12" width="8.69140625" style="51" customWidth="1"/>
-    <col min="13" max="16384" width="8.69140625" style="51"/>
+    <col min="1" max="1" width="12.23046875" style="50" customWidth="1"/>
+    <col min="2" max="2" width="46.53515625" style="50" customWidth="1"/>
+    <col min="3" max="3" width="22.4609375" style="50" customWidth="1"/>
+    <col min="4" max="4" width="8.4609375" style="50" customWidth="1"/>
+    <col min="5" max="5" width="43.53515625" style="50" customWidth="1"/>
+    <col min="6" max="6" width="50.4609375" style="50" customWidth="1"/>
+    <col min="7" max="7" width="23.84375" style="50" customWidth="1"/>
+    <col min="8" max="8" width="54.4609375" style="50" customWidth="1"/>
+    <col min="9" max="9" width="20.15234375" style="56" customWidth="1"/>
+    <col min="10" max="12" width="8.69140625" style="50" customWidth="1"/>
+    <col min="13" max="16384" width="8.69140625" style="50"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="38" customFormat="1" ht="18.45" customHeight="1">
-      <c r="A1" s="38" t="s">
+    <row r="1" spans="1:9" s="37" customFormat="1" ht="18.45" customHeight="1">
+      <c r="A1" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="37" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" s="39"/>
+      <c r="E1" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="38" t="s">
+      <c r="F1" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="C1" s="39" t="s">
+      <c r="G1" s="38" t="s">
         <v>91</v>
       </c>
-      <c r="D1" s="40"/>
-      <c r="E1" s="39" t="s">
+      <c r="H1" s="38" t="s">
         <v>92</v>
       </c>
-      <c r="F1" s="39" t="s">
+      <c r="I1" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="G1" s="39" t="s">
+    </row>
+    <row r="2" spans="1:9" s="37" customFormat="1" ht="18.45" customHeight="1">
+      <c r="A2" s="41" t="s">
         <v>94</v>
       </c>
-      <c r="H1" s="39" t="s">
+      <c r="B2" s="41" t="s">
         <v>95</v>
       </c>
-      <c r="I1" s="41" t="s">
+      <c r="C2" s="26" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" s="38" customFormat="1" ht="18.45" customHeight="1">
-      <c r="A2" s="42" t="s">
-        <v>97</v>
-      </c>
-      <c r="B2" s="42" t="s">
-        <v>98</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>99</v>
-      </c>
-      <c r="D2" s="43" t="str">
+      <c r="D2" s="42" t="str">
         <f t="shared" ref="D2:D14" si="0">HYPERLINK(CONCATENATE("https://nvd.nist.gov/vuln/detail/", C2), "🔗")</f>
         <v>🔗</v>
       </c>
-      <c r="E2" s="42" t="s">
+      <c r="E2" s="41" t="s">
+        <v>97</v>
+      </c>
+      <c r="F2" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="G2" s="41" t="s">
+        <v>99</v>
+      </c>
+      <c r="H2" s="41" t="s">
         <v>100</v>
       </c>
-      <c r="F2" s="24" t="s">
+      <c r="I2" s="41"/>
+    </row>
+    <row r="3" spans="1:9" ht="30.9" customHeight="1">
+      <c r="A3" s="43" t="s">
         <v>101</v>
       </c>
-      <c r="G2" s="42" t="s">
+      <c r="B3" s="44" t="s">
         <v>102</v>
       </c>
-      <c r="H2" s="42" t="s">
+      <c r="C3" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="I2" s="42"/>
-    </row>
-    <row r="3" spans="1:9" ht="30.9" customHeight="1">
-      <c r="A3" s="44" t="s">
-        <v>104</v>
-      </c>
-      <c r="B3" s="45" t="s">
-        <v>105</v>
-      </c>
-      <c r="C3" s="46" t="s">
-        <v>106</v>
-      </c>
-      <c r="D3" s="47" t="str">
+      <c r="D3" s="46" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E3" s="48" t="s">
+      <c r="E3" s="47" t="s">
+        <v>104</v>
+      </c>
+      <c r="F3" s="48" t="s">
+        <v>105</v>
+      </c>
+      <c r="G3" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="H3" s="49" t="s">
         <v>107</v>
       </c>
-      <c r="F3" s="49" t="s">
+      <c r="I3" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="G3" s="48" t="s">
+    </row>
+    <row r="4" spans="1:9" s="37" customFormat="1" ht="18.45" customHeight="1">
+      <c r="A4" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" s="41" t="s">
         <v>109</v>
       </c>
-      <c r="H3" s="50" t="s">
+      <c r="C4" s="26" t="s">
         <v>110</v>
       </c>
-      <c r="I3" s="42" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" s="38" customFormat="1" ht="18.45" customHeight="1">
-      <c r="A4" s="42" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" s="42" t="s">
-        <v>112</v>
-      </c>
-      <c r="C4" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="D4" s="43" t="str">
+      <c r="D4" s="42" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E4" s="42" t="s">
+      <c r="E4" s="41" t="s">
+        <v>111</v>
+      </c>
+      <c r="F4" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="G4" s="41" t="s">
+        <v>99</v>
+      </c>
+      <c r="H4" s="41" t="s">
+        <v>113</v>
+      </c>
+      <c r="I4" s="41"/>
+    </row>
+    <row r="5" spans="1:9" s="37" customFormat="1" ht="30.9" customHeight="1">
+      <c r="A5" s="43" t="s">
+        <v>101</v>
+      </c>
+      <c r="B5" s="44" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="45" t="s">
         <v>114</v>
       </c>
-      <c r="F4" s="24" t="s">
-        <v>115</v>
-      </c>
-      <c r="G4" s="42" t="s">
-        <v>102</v>
-      </c>
-      <c r="H4" s="42" t="s">
-        <v>116</v>
-      </c>
-      <c r="I4" s="42"/>
-    </row>
-    <row r="5" spans="1:9" s="38" customFormat="1" ht="30.9" customHeight="1">
-      <c r="A5" s="44" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" s="45" t="s">
-        <v>105</v>
-      </c>
-      <c r="C5" s="46" t="s">
-        <v>117</v>
-      </c>
-      <c r="D5" s="47" t="str">
+      <c r="D5" s="46" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E5" s="48" t="s">
-        <v>107</v>
-      </c>
-      <c r="F5" s="49" t="s">
+      <c r="E5" s="47" t="s">
+        <v>104</v>
+      </c>
+      <c r="F5" s="48" t="s">
+        <v>105</v>
+      </c>
+      <c r="G5" s="47" t="s">
+        <v>115</v>
+      </c>
+      <c r="H5" s="49" t="s">
+        <v>105</v>
+      </c>
+      <c r="I5" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="G5" s="48" t="s">
-        <v>118</v>
-      </c>
-      <c r="H5" s="50" t="s">
-        <v>108</v>
-      </c>
-      <c r="I5" s="42" t="s">
-        <v>111</v>
-      </c>
     </row>
     <row r="6" spans="1:9" ht="77.150000000000006" customHeight="1">
-      <c r="A6" s="44" t="s">
-        <v>104</v>
-      </c>
-      <c r="B6" s="45" t="s">
-        <v>119</v>
-      </c>
-      <c r="C6" s="46" t="s">
-        <v>120</v>
-      </c>
-      <c r="D6" s="47" t="str">
+      <c r="A6" s="43" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6" s="45" t="s">
+        <v>117</v>
+      </c>
+      <c r="D6" s="46" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E6" s="48" t="s">
+      <c r="E6" s="47" t="s">
+        <v>118</v>
+      </c>
+      <c r="F6" s="48" t="s">
+        <v>119</v>
+      </c>
+      <c r="G6" s="47" t="s">
+        <v>120</v>
+      </c>
+      <c r="H6" s="49" t="s">
         <v>121</v>
       </c>
-      <c r="F6" s="49" t="s">
+      <c r="I6" s="41"/>
+    </row>
+    <row r="7" spans="1:9" ht="61.75" customHeight="1">
+      <c r="A7" s="43" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="C7" s="45" t="s">
         <v>122</v>
       </c>
-      <c r="G6" s="48" t="s">
-        <v>123</v>
-      </c>
-      <c r="H6" s="50" t="s">
-        <v>124</v>
-      </c>
-      <c r="I6" s="42"/>
-    </row>
-    <row r="7" spans="1:9" ht="61.75" customHeight="1">
-      <c r="A7" s="44" t="s">
-        <v>104</v>
-      </c>
-      <c r="B7" s="45" t="s">
-        <v>119</v>
-      </c>
-      <c r="C7" s="46" t="s">
-        <v>125</v>
-      </c>
-      <c r="D7" s="47" t="str">
+      <c r="D7" s="46" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E7" s="48" t="s">
-        <v>107</v>
-      </c>
-      <c r="F7" s="52" t="s">
-        <v>126</v>
-      </c>
-      <c r="G7" s="48" t="s">
+      <c r="E7" s="47" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7" s="51" t="s">
         <v>123</v>
       </c>
-      <c r="H7" s="48" t="s">
-        <v>127</v>
-      </c>
-      <c r="I7" s="42" t="s">
-        <v>111</v>
+      <c r="G7" s="47" t="s">
+        <v>120</v>
+      </c>
+      <c r="H7" s="47" t="s">
+        <v>124</v>
+      </c>
+      <c r="I7" s="41" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.45" customHeight="1">
-      <c r="A8" s="42" t="s">
-        <v>104</v>
-      </c>
-      <c r="B8" s="42" t="s">
-        <v>112</v>
-      </c>
-      <c r="C8" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="D8" s="43" t="str">
+      <c r="A8" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="41" t="s">
+        <v>109</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="D8" s="42" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="41" t="s">
+        <v>126</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="G8" s="41" t="s">
+        <v>128</v>
+      </c>
+      <c r="H8" s="52" t="s">
         <v>129</v>
       </c>
-      <c r="F8" s="24" t="s">
+      <c r="I8" s="41"/>
+    </row>
+    <row r="9" spans="1:9" ht="30.9" customHeight="1">
+      <c r="A9" s="43" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>102</v>
+      </c>
+      <c r="C9" s="45" t="s">
         <v>130</v>
       </c>
-      <c r="G8" s="42" t="s">
-        <v>131</v>
-      </c>
-      <c r="H8" s="53" t="s">
-        <v>132</v>
-      </c>
-      <c r="I8" s="42"/>
-    </row>
-    <row r="9" spans="1:9" ht="30.9" customHeight="1">
-      <c r="A9" s="44" t="s">
-        <v>104</v>
-      </c>
-      <c r="B9" s="45" t="s">
-        <v>105</v>
-      </c>
-      <c r="C9" s="46" t="s">
-        <v>133</v>
-      </c>
-      <c r="D9" s="47" t="str">
+      <c r="D9" s="46" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E9" s="48" t="s">
-        <v>107</v>
-      </c>
-      <c r="F9" s="49" t="s">
+      <c r="E9" s="47" t="s">
+        <v>104</v>
+      </c>
+      <c r="F9" s="48" t="s">
+        <v>131</v>
+      </c>
+      <c r="G9" s="47" t="s">
+        <v>132</v>
+      </c>
+      <c r="H9" s="49" t="s">
+        <v>133</v>
+      </c>
+      <c r="I9" s="41" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="92.6" customHeight="1">
+      <c r="A10" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="B10" s="41" t="s">
+        <v>109</v>
+      </c>
+      <c r="C10" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="G9" s="48" t="s">
-        <v>135</v>
-      </c>
-      <c r="H9" s="50" t="s">
-        <v>136</v>
-      </c>
-      <c r="I9" s="42" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="92.6" customHeight="1">
-      <c r="A10" s="42" t="s">
-        <v>104</v>
-      </c>
-      <c r="B10" s="42" t="s">
-        <v>112</v>
-      </c>
-      <c r="C10" s="27" t="s">
-        <v>137</v>
-      </c>
-      <c r="D10" s="43" t="str">
+      <c r="D10" s="42" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E10" s="42" t="s">
+      <c r="E10" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>136</v>
+      </c>
+      <c r="G10" s="41" t="s">
+        <v>137</v>
+      </c>
+      <c r="H10" s="52" t="s">
         <v>138</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="I10" s="41"/>
+    </row>
+    <row r="11" spans="1:9" ht="77.150000000000006" customHeight="1">
+      <c r="A11" s="53" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" s="45" t="s">
         <v>139</v>
       </c>
-      <c r="G10" s="42" t="s">
-        <v>140</v>
-      </c>
-      <c r="H10" s="53" t="s">
-        <v>141</v>
-      </c>
-      <c r="I10" s="42"/>
-    </row>
-    <row r="11" spans="1:9" ht="77.150000000000006" customHeight="1">
-      <c r="A11" s="54" t="s">
-        <v>97</v>
-      </c>
-      <c r="B11" s="45" t="s">
-        <v>119</v>
-      </c>
-      <c r="C11" s="46" t="s">
-        <v>142</v>
-      </c>
-      <c r="D11" s="47" t="str">
+      <c r="D11" s="46" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E11" s="48" t="s">
-        <v>107</v>
-      </c>
-      <c r="F11" s="49" t="s">
+      <c r="E11" s="47" t="s">
+        <v>104</v>
+      </c>
+      <c r="F11" s="48" t="s">
+        <v>105</v>
+      </c>
+      <c r="G11" s="47" t="s">
+        <v>140</v>
+      </c>
+      <c r="H11" s="49" t="s">
+        <v>141</v>
+      </c>
+      <c r="I11" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="G11" s="48" t="s">
-        <v>143</v>
-      </c>
-      <c r="H11" s="50" t="s">
-        <v>144</v>
-      </c>
-      <c r="I11" s="42" t="s">
-        <v>111</v>
-      </c>
     </row>
     <row r="12" spans="1:9" ht="30.9" customHeight="1">
-      <c r="A12" s="42" t="s">
-        <v>104</v>
-      </c>
-      <c r="B12" s="45" t="s">
-        <v>105</v>
-      </c>
-      <c r="C12" s="27" t="s">
-        <v>145</v>
-      </c>
-      <c r="D12" s="43" t="str">
+      <c r="A12" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" s="44" t="s">
+        <v>102</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>142</v>
+      </c>
+      <c r="D12" s="42" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E12" s="42" t="s">
+      <c r="E12" s="41" t="s">
+        <v>143</v>
+      </c>
+      <c r="F12" s="52" t="s">
+        <v>144</v>
+      </c>
+      <c r="G12" s="41" t="s">
+        <v>145</v>
+      </c>
+      <c r="H12" s="52" t="s">
         <v>146</v>
       </c>
-      <c r="F12" s="53" t="s">
+      <c r="I12" s="41"/>
+    </row>
+    <row r="13" spans="1:9" ht="46.3" customHeight="1">
+      <c r="A13" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="B13" s="44" t="s">
+        <v>116</v>
+      </c>
+      <c r="C13" s="26" t="s">
         <v>147</v>
       </c>
-      <c r="G12" s="42" t="s">
-        <v>148</v>
-      </c>
-      <c r="H12" s="53" t="s">
-        <v>149</v>
-      </c>
-      <c r="I12" s="42"/>
-    </row>
-    <row r="13" spans="1:9" ht="46.3" customHeight="1">
-      <c r="A13" s="42" t="s">
-        <v>104</v>
-      </c>
-      <c r="B13" s="45" t="s">
-        <v>119</v>
-      </c>
-      <c r="C13" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="D13" s="43" t="str">
+      <c r="D13" s="42" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E13" s="42" t="s">
+      <c r="E13" s="41" t="s">
+        <v>148</v>
+      </c>
+      <c r="F13" s="52" t="s">
+        <v>149</v>
+      </c>
+      <c r="G13" s="41" t="s">
+        <v>150</v>
+      </c>
+      <c r="H13" s="52" t="s">
         <v>151</v>
       </c>
-      <c r="F13" s="53" t="s">
+      <c r="I13" s="41"/>
+    </row>
+    <row r="14" spans="1:9" ht="46.3" customHeight="1">
+      <c r="A14" s="41" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" s="41" t="s">
         <v>152</v>
       </c>
-      <c r="G13" s="42" t="s">
+      <c r="C14" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="H13" s="53" t="s">
-        <v>154</v>
-      </c>
-      <c r="I13" s="42"/>
-    </row>
-    <row r="14" spans="1:9" ht="46.3" customHeight="1">
-      <c r="A14" s="42" t="s">
-        <v>97</v>
-      </c>
-      <c r="B14" s="42" t="s">
-        <v>155</v>
-      </c>
-      <c r="C14" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="D14" s="43" t="str">
+      <c r="D14" s="42" t="str">
         <f t="shared" si="0"/>
         <v>🔗</v>
       </c>
-      <c r="E14" s="42" t="s">
-        <v>151</v>
-      </c>
-      <c r="F14" s="53" t="s">
-        <v>157</v>
-      </c>
-      <c r="G14" s="42" t="s">
-        <v>153</v>
-      </c>
-      <c r="H14" s="53" t="s">
-        <v>158</v>
-      </c>
-      <c r="I14" s="42"/>
+      <c r="E14" s="41" t="s">
+        <v>148</v>
+      </c>
+      <c r="F14" s="52" t="s">
+        <v>154</v>
+      </c>
+      <c r="G14" s="41" t="s">
+        <v>150</v>
+      </c>
+      <c r="H14" s="52" t="s">
+        <v>155</v>
+      </c>
+      <c r="I14" s="41"/>
     </row>
     <row r="17" spans="1:2" ht="15.9" customHeight="1">
-      <c r="A17" s="55"/>
-      <c r="B17" s="56"/>
+      <c r="A17" s="54"/>
+      <c r="B17" s="55"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -10589,17 +10592,17 @@
   <sheetData>
     <row r="1" spans="1:1" ht="14.15" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="14.15" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:1" ht="14.15" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="14.15" customHeight="1">
@@ -10619,12 +10622,12 @@
     </row>
     <row r="7" spans="1:1" ht="14.15" customHeight="1">
       <c r="A7" s="10" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="14.15" customHeight="1">
       <c r="A8" s="10" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="14.15" customHeight="1">

</xml_diff>